<commit_message>
Rename board to bulletin and fix bulletin posting bugs
- Rename all board references to bulletin (closes #314)

- Fix bulletin post success not returning to previous screen

- Fix URL encoding issues in HTTP requests

- Add proper exception handling for HTTP GET/POST operations
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75FB762C-9FDB-4887-BE64-C23C0B7C51AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5999AC1-847B-4EC2-9E18-9537ECA2A05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="regex" sheetId="1" r:id="rId1"/>
@@ -394,9 +394,6 @@
     <t>MESSAGE_ASSET_CLASS_LOADED</t>
   </si>
   <si>
-    <t>MESSAGE_ASSET_BOARD_LOADED</t>
-  </si>
-  <si>
     <t>MESSAGE_ASSET_MAP_ALL_LOADED</t>
   </si>
   <si>
@@ -445,9 +442,6 @@
     <t>MESSAGE_ASSET_CLASS_ALL_LOADED</t>
   </si>
   <si>
-    <t>MESSAGE_ASSET_BOARD_ALL_LOADED</t>
-  </si>
-  <si>
     <t>MESSAGE_ASSET_INVALID_SEX</t>
   </si>
   <si>
@@ -596,27 +590,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MESSAGE_BOARD_WRITE</t>
-  </si>
-  <si>
-    <t>MESSAGE_BOARD_ARTICLE_NOT_EXIST</t>
-  </si>
-  <si>
-    <t>MESSAGE_BOARD_SECTION_NOT_EXIST</t>
-  </si>
-  <si>
-    <t>MESSAGE_BOARD_NOT_AUTH</t>
-  </si>
-  <si>
-    <t>MESSAGE_BOARD_SUCCESS_DELETE</t>
-  </si>
-  <si>
-    <t>MESSAGE_BOARD_TOO_LONG_TITLE</t>
-  </si>
-  <si>
-    <t>MESSAGE_BOARD_TOO_LONG_CONTENTS</t>
-  </si>
-  <si>
     <t>MESSAGE_DOOR_OPEN</t>
   </si>
   <si>
@@ -849,10 +822,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MESSAGE_WRITE_BOARD_FAILED</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>게시글 작성 실패</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1167,6 +1136,36 @@
   <si>
     <t>RETRIEVE_ITEM</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MESSAGE_ASSET_BULLETIN_LOADED</t>
+  </si>
+  <si>
+    <t>MESSAGE_ASSET_BULLETIN_ALL_LOADED</t>
+  </si>
+  <si>
+    <t>MESSAGE_BULLETIN_WRITE</t>
+  </si>
+  <si>
+    <t>MESSAGE_BULLETIN_ARTICLE_NOT_EXIST</t>
+  </si>
+  <si>
+    <t>MESSAGE_BULLETIN_SECTION_NOT_EXIST</t>
+  </si>
+  <si>
+    <t>MESSAGE_BULLETIN_NOT_AUTH</t>
+  </si>
+  <si>
+    <t>MESSAGE_BULLETIN_SUCCESS_DELETE</t>
+  </si>
+  <si>
+    <t>MESSAGE_BULLETIN_TOO_LONG_TITLE</t>
+  </si>
+  <si>
+    <t>MESSAGE_BULLETIN_TOO_LONG_CONTENTS</t>
+  </si>
+  <si>
+    <t>MESSAGE_WRITE_BULLETIN_FAILED</t>
   </si>
 </sst>
 </file>
@@ -1651,7 +1650,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>0</v>
@@ -1665,7 +1664,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>359</v>
+        <v>349</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>0</v>
@@ -1716,7 +1715,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>350</v>
+        <v>340</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -1791,7 +1790,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>0</v>
@@ -1800,12 +1799,12 @@
         <v>1</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>0</v>
@@ -1814,7 +1813,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -1835,13 +1834,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>351</v>
+        <v>341</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
       <c r="D1" s="3">
         <v>6.9444444444444447E-4</v>
@@ -1864,13 +1863,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>353</v>
+        <v>343</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>354</v>
+        <v>344</v>
       </c>
       <c r="D1" s="4">
         <v>0.05</v>
@@ -1878,27 +1877,27 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>355</v>
+        <v>345</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>354</v>
+        <v>344</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
       <c r="D3" s="3">
         <v>2.0833333333333332E-2</v>
@@ -1921,86 +1920,86 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -2023,7 +2022,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -2037,7 +2036,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
@@ -2051,7 +2050,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>0</v>
@@ -2065,7 +2064,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>0</v>
@@ -2079,7 +2078,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>0</v>
@@ -2093,7 +2092,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>0</v>
@@ -2107,7 +2106,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>0</v>
@@ -2121,7 +2120,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>0</v>
@@ -2135,7 +2134,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>0</v>
@@ -2149,7 +2148,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>0</v>
@@ -2163,7 +2162,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>0</v>
@@ -2186,7 +2185,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -2200,7 +2199,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -2214,7 +2213,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -2228,7 +2227,7 @@
         <v>1</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -2242,7 +2241,7 @@
         <v>1</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -2256,7 +2255,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -2270,7 +2269,7 @@
         <v>1</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -2284,7 +2283,7 @@
         <v>1</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -2298,7 +2297,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -2312,7 +2311,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -2326,7 +2325,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -2340,7 +2339,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -2354,7 +2353,7 @@
         <v>1</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -2368,7 +2367,7 @@
         <v>1</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -2382,7 +2381,7 @@
         <v>1</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -2396,12 +2395,12 @@
         <v>1</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>120</v>
+        <v>350</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>0</v>
@@ -2410,12 +2409,12 @@
         <v>1</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>0</v>
@@ -2424,12 +2423,12 @@
         <v>1</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>0</v>
@@ -2438,12 +2437,12 @@
         <v>1</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>0</v>
@@ -2452,12 +2451,12 @@
         <v>1</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>0</v>
@@ -2466,12 +2465,12 @@
         <v>1</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>0</v>
@@ -2480,12 +2479,12 @@
         <v>1</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>0</v>
@@ -2494,12 +2493,12 @@
         <v>1</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>0</v>
@@ -2508,12 +2507,12 @@
         <v>1</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>0</v>
@@ -2522,12 +2521,12 @@
         <v>1</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>0</v>
@@ -2536,12 +2535,12 @@
         <v>1</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>0</v>
@@ -2550,12 +2549,12 @@
         <v>1</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>0</v>
@@ -2564,12 +2563,12 @@
         <v>1</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>0</v>
@@ -2578,12 +2577,12 @@
         <v>1</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>0</v>
@@ -2592,12 +2591,12 @@
         <v>1</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>0</v>
@@ -2606,12 +2605,12 @@
         <v>1</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>0</v>
@@ -2620,12 +2619,12 @@
         <v>1</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>0</v>
@@ -2634,12 +2633,12 @@
         <v>1</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>137</v>
+        <v>351</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>0</v>
@@ -2648,12 +2647,12 @@
         <v>1</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>0</v>
@@ -2667,7 +2666,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>0</v>
@@ -2681,7 +2680,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>0</v>
@@ -2695,7 +2694,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>0</v>
@@ -2709,7 +2708,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>0</v>
@@ -2723,7 +2722,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>0</v>
@@ -2737,7 +2736,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>0</v>
@@ -2751,7 +2750,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>0</v>
@@ -2765,7 +2764,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>0</v>
@@ -2779,7 +2778,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>0</v>
@@ -2793,7 +2792,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>0</v>
@@ -2807,7 +2806,7 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>0</v>
@@ -2821,7 +2820,7 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>0</v>
@@ -2835,7 +2834,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>0</v>
@@ -2849,7 +2848,7 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>0</v>
@@ -2863,7 +2862,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>0</v>
@@ -2877,7 +2876,7 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>0</v>
@@ -2891,7 +2890,7 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>0</v>
@@ -2905,7 +2904,7 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>0</v>
@@ -2914,12 +2913,12 @@
         <v>1</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>0</v>
@@ -2933,7 +2932,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>0</v>
@@ -2947,7 +2946,7 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>0</v>
@@ -2961,7 +2960,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>0</v>
@@ -2975,7 +2974,7 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>0</v>
@@ -2989,7 +2988,7 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>0</v>
@@ -3003,7 +3002,7 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>0</v>
@@ -3017,7 +3016,7 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>0</v>
@@ -3031,7 +3030,7 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>0</v>
@@ -3045,7 +3044,7 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>0</v>
@@ -3059,7 +3058,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>0</v>
@@ -3073,7 +3072,7 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>0</v>
@@ -3087,7 +3086,7 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>0</v>
@@ -3101,7 +3100,7 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>0</v>
@@ -3115,7 +3114,7 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>0</v>
@@ -3129,7 +3128,7 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>0</v>
@@ -3143,7 +3142,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>0</v>
@@ -3157,7 +3156,7 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>0</v>
@@ -3171,7 +3170,7 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>0</v>
@@ -3185,7 +3184,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>0</v>
@@ -3199,7 +3198,7 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>0</v>
@@ -3213,7 +3212,7 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>0</v>
@@ -3227,7 +3226,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>0</v>
@@ -3241,7 +3240,7 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>0</v>
@@ -3255,7 +3254,7 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>0</v>
@@ -3269,7 +3268,7 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>0</v>
@@ -3283,7 +3282,7 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>0</v>
@@ -3297,7 +3296,7 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>0</v>
@@ -3311,7 +3310,7 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>0</v>
@@ -3325,7 +3324,7 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>0</v>
@@ -3339,7 +3338,7 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>0</v>
@@ -3353,7 +3352,7 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>0</v>
@@ -3367,7 +3366,7 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>0</v>
@@ -3381,7 +3380,7 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>0</v>
@@ -3395,7 +3394,7 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
-        <v>187</v>
+        <v>352</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>0</v>
@@ -3409,7 +3408,7 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
-        <v>188</v>
+        <v>353</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>0</v>
@@ -3423,7 +3422,7 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
-        <v>189</v>
+        <v>354</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>0</v>
@@ -3437,7 +3436,7 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
-        <v>190</v>
+        <v>355</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>0</v>
@@ -3451,7 +3450,7 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
-        <v>191</v>
+        <v>356</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>0</v>
@@ -3465,7 +3464,7 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
-        <v>192</v>
+        <v>357</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>0</v>
@@ -3479,7 +3478,7 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
-        <v>193</v>
+        <v>358</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>0</v>
@@ -3493,7 +3492,7 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>0</v>
@@ -3507,7 +3506,7 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>0</v>
@@ -3521,7 +3520,7 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>0</v>
@@ -3535,7 +3534,7 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>0</v>
@@ -3549,7 +3548,7 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>0</v>
@@ -3563,7 +3562,7 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>0</v>
@@ -3577,7 +3576,7 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>0</v>
@@ -3586,12 +3585,12 @@
         <v>1</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>0</v>
@@ -3600,12 +3599,12 @@
         <v>1</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>0</v>
@@ -3614,12 +3613,12 @@
         <v>1</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>0</v>
@@ -3628,12 +3627,12 @@
         <v>1</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
-        <v>267</v>
+        <v>359</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>0</v>
@@ -3642,12 +3641,12 @@
         <v>1</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>0</v>
@@ -3656,12 +3655,12 @@
         <v>1</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>0</v>
@@ -3670,12 +3669,12 @@
         <v>1</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>0</v>
@@ -3684,12 +3683,12 @@
         <v>1</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>0</v>
@@ -3698,12 +3697,12 @@
         <v>1</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>0</v>
@@ -3712,12 +3711,12 @@
         <v>1</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>0</v>
@@ -3726,12 +3725,12 @@
         <v>1</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>0</v>
@@ -3740,12 +3739,12 @@
         <v>1</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>0</v>
@@ -3754,12 +3753,12 @@
         <v>1</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>0</v>
@@ -3768,12 +3767,12 @@
         <v>1</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>0</v>
@@ -3782,12 +3781,12 @@
         <v>1</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>0</v>
@@ -3796,12 +3795,12 @@
         <v>1</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>0</v>
@@ -3810,12 +3809,12 @@
         <v>1</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>0</v>
@@ -3824,12 +3823,12 @@
         <v>1</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>0</v>
@@ -3838,12 +3837,12 @@
         <v>1</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>0</v>
@@ -3852,12 +3851,12 @@
         <v>1</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>0</v>
@@ -3866,12 +3865,12 @@
         <v>1</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>0</v>
@@ -3880,12 +3879,12 @@
         <v>1</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>0</v>
@@ -3894,12 +3893,12 @@
         <v>1</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>0</v>
@@ -3908,12 +3907,12 @@
         <v>1</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>0</v>
@@ -3922,12 +3921,12 @@
         <v>1</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>0</v>
@@ -3936,12 +3935,12 @@
         <v>1</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>0</v>
@@ -3950,12 +3949,12 @@
         <v>1</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>0</v>
@@ -3964,12 +3963,12 @@
         <v>1</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>0</v>
@@ -3978,12 +3977,12 @@
         <v>1</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>0</v>
@@ -3992,12 +3991,12 @@
         <v>1</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>0</v>
@@ -4006,12 +4005,12 @@
         <v>1</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>0</v>
@@ -4020,12 +4019,12 @@
         <v>1</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="B144" s="2" t="s">
         <v>0</v>
@@ -4034,12 +4033,12 @@
         <v>1</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="B145" s="2" t="s">
         <v>0</v>
@@ -4048,12 +4047,12 @@
         <v>1</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>0</v>
@@ -4062,12 +4061,12 @@
         <v>1</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="B147" s="2" t="s">
         <v>0</v>
@@ -4076,12 +4075,12 @@
         <v>1</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>0</v>
@@ -4090,12 +4089,12 @@
         <v>1</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="B149" s="2" t="s">
         <v>0</v>
@@ -4104,12 +4103,12 @@
         <v>1</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>0</v>
@@ -4118,12 +4117,12 @@
         <v>1</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>343</v>
+        <v>333</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>0</v>
@@ -4132,7 +4131,7 @@
         <v>1</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -4152,16 +4151,16 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: remove BOW item type and improve equipment tests
- Remove BOW item type support from game engine
- Delete bow.cpp implementation file
- Remove bow class from item.h header
- Clean up bow references in model.item.cpp
- Refactor equipment test scenarios for better maintainability
- Improve bot chat logging in equipment tests
- Update data tables and model configurations
- Simplify test logic with better error handling
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5999AC1-847B-4EC2-9E18-9537ECA2A05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A0CE5B9-CA94-442A-86DC-CFFEB046D1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="362">
   <si>
     <t>server</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1166,6 +1166,14 @@
   </si>
   <si>
     <t>MESSAGE_WRITE_BULLETIN_FAILED</t>
+  </si>
+  <si>
+    <t>MESSAGE_NO_RECIPE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조합할 수 없습니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -2010,7 +2018,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BFB54FE-6D3B-49A4-815A-82E992FE6C32}">
-  <dimension ref="A1:D151"/>
+  <dimension ref="A1:D152"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.5" style="2" bestFit="1" customWidth="1"/>
@@ -4132,6 +4140,20 @@
       </c>
       <c r="D151" s="2" t="s">
         <v>335</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A152" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>361</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: separate leave and kick functionality for clan and group
- Split leave_clan_member into leave and kick functions
- Add kick_clan_member and kick_group_member builtin functions
- Implement permission checks for clan and group expulsion
- Update FlatBuffer protocols to support separate kick operations
- Add AMQP handlers for kick notifications
- Update wiki documentation for new kick functions
- Refactor controllers to handle leave vs kick logic separately
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A0CE5B9-CA94-442A-86DC-CFFEB046D1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31ABAC2D-0EC4-4091-B733-DB33F6F2C94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="regex" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="death_penalty" sheetId="6" r:id="rId3"/>
     <sheet name="item" sheetId="4" r:id="rId4"/>
     <sheet name="string" sheetId="2" r:id="rId5"/>
-    <sheet name="mob" sheetId="3" r:id="rId6"/>
+    <sheet name="clan" sheetId="7" r:id="rId6"/>
+    <sheet name="mob" sheetId="3" r:id="rId7"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="365">
   <si>
     <t>server</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1173,6 +1174,17 @@
   </si>
   <si>
     <t>조합할 수 없습니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MIN_KICKABLE_POSITION</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DEPUTY</t>
+  </si>
+  <si>
+    <t>CLAN_POSITION</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -4164,6 +4176,35 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2413674-7644-40A9-9F6B-053B0D52D095}">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>364</v>
+      </c>
+      <c r="D1" t="s">
+        <v>363</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71AA2139-4412-4459-975E-C6152019FA56}">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
feat: implement invitation-based clan join system with role-based permissions
- Refactor clan join system to use inviter/invitee model instead of direct join
- Add comprehensive permission checks for clan actions (invite, kick, change role)
- Update FlatBuffer schemas to support new invitation-based join process
- Implement role-based privilege system with CLAN_ROLE enum
- Add proper error handling and validation in C# APIs
- Update C++ builtin functions to support new join mechanism
- Modify Lua scripts to use new clan:join(inviter, invitee) signature
- Add distributed locking and transaction safety for clan operations
- Update documentation and wiki to reflect new system architecture
- Replace hardcoded position checks with configurable privilege constants
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31ABAC2D-0EC4-4091-B733-DB33F6F2C94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F6734A-70F3-497A-B8D7-192FEB784559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="regex" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,8 @@
     <sheet name="death_penalty" sheetId="6" r:id="rId3"/>
     <sheet name="item" sheetId="4" r:id="rId4"/>
     <sheet name="string" sheetId="2" r:id="rId5"/>
-    <sheet name="clan" sheetId="7" r:id="rId6"/>
-    <sheet name="mob" sheetId="3" r:id="rId7"/>
+    <sheet name="mob" sheetId="3" r:id="rId6"/>
+    <sheet name="clan" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="367">
   <si>
     <t>server</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1177,14 +1177,23 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MIN_KICKABLE_POSITION</t>
+    <t>CLAN_ROLE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>DEPUTY</t>
-  </si>
-  <si>
-    <t>CLAN_POSITION</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MINIMUM_INVITE_PRIVILEGE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MINIMUM_KICK_PRIVILEGE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MINIMUM_CHANGE_ROLE_PRIVILEGE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1268,7 +1277,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1284,7 +1293,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -4176,35 +4185,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2413674-7644-40A9-9F6B-053B0D52D095}">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="24.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>362</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>364</v>
-      </c>
-      <c r="D1" t="s">
-        <v>363</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71AA2139-4412-4459-975E-C6152019FA56}">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -4230,4 +4210,63 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5047E650-3765-47B1-A7FE-DA9F7A8550D3}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="31.625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="5"/>
+    <col min="3" max="3" width="10.25" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>363</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement clan title change functionality
- Add clan title change methods to game_bot (change_clan_title)
- Implement clan title change test scenario with role-based permission validation
- Update clan builtin functions to support title changes with privilege checks
- Modify HTTP API to use changer-based clan identification instead of explicit clan ID
- Add MinimumChangeTitlePrivilege constant for title change permission control
- Update FlatBuffer protocol to support new title change request structure
- Refactor clan test scenarios to use new bot methods for better maintainability
- Update wiki documentation to reflect new function signatures and parameters
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F6734A-70F3-497A-B8D7-192FEB784559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C37F1CF-3438-4902-A6DD-51009AE01BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="regex" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="369">
   <si>
     <t>server</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1194,6 +1194,14 @@
   </si>
   <si>
     <t>MINIMUM_CHANGE_ROLE_PRIVILEGE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MINIMUM_CHANGE_TITLE_PRIVILEGE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MASTER</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1277,7 +1285,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1293,7 +1301,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -4214,7 +4222,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5047E650-3765-47B1-A7FE-DA9F7A8550D3}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.625" style="5" bestFit="1" customWidth="1"/>
@@ -4265,6 +4273,20 @@
         <v>363</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>368</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: implement mail system level requirements and button improvements
- Add MAIL_BUTTON_ENABLE::UP enum value
- Add mail const class with REQUIRED_LEVEL and COUNT_PER_PAGE
- Update bulletin handler to use level-based mail button logic
- Replace hardcoded values with const values
- Fix mail button flag logic for different scenarios
- Update Excel configuration tables
- Update model generation timestamp
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C37F1CF-3438-4902-A6DD-51009AE01BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28F3039-5446-40E4-B934-0F685D2B3B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="8" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="regex" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,8 @@
     <sheet name="string" sheetId="2" r:id="rId5"/>
     <sheet name="mob" sheetId="3" r:id="rId6"/>
     <sheet name="clan" sheetId="7" r:id="rId7"/>
+    <sheet name="mail" sheetId="8" r:id="rId8"/>
+    <sheet name="script" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="379">
   <si>
     <t>server</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1202,6 +1204,46 @@
   </si>
   <si>
     <t>MASTER</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>uint8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>COUNT_PER_PAGE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>REQUIRED_LEVEL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>F1_EVENT_SCRIPT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>F2_EVENT_SCRIPT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>F1_EVENT_FUNC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scripts/server.lua</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ON_F1_EVENT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>F2_EVENT_FUNC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ON_F2_EVENT</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -4291,4 +4333,120 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25A28286-3AEF-42D4-85D1-723078A774E6}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="D1" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="D2" s="2">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49D81130-7A86-4FD0-BE88-6F2B508E57F2}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="9" style="2"/>
+    <col min="4" max="4" width="18.625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: improve marketplace listing system
- Remove expire_hours from List request protocol
- Add marketplace constants (page_size, expire_time, listing_limit) to model
- Add MARKETPLACE_LISTING_LIMIT_EXCEEDED error code
- Refactor status handling to use ListingState enum instead of byte
- Add listing limit validation per seller
- Enhance MySql extension to support enum types
- Remove marketplace configuration from appsettings and pulumi
- Update expiration handling to use TimeSpan
- Improve transaction handling in search operations
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F737DA1E-84EB-4AA1-929E-1A1823DD18B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB4FF51C-BA1E-430E-BDE5-D49C6A93FC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="regex" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="83">
   <si>
     <t>server</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -307,6 +307,26 @@
   </si>
   <si>
     <t>listing_fee</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>page_size</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>int</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>expire_time</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3.00:00:00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>listing_limit</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -390,7 +410,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -406,7 +426,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -1180,10 +1200,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5478E627-A9E2-4CC4-9690-22D3BFBD3A42}">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1198,6 +1219,48 @@
       </c>
       <c r="D1" s="1" t="s">
         <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="5">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add NPC interaction validation in Lua script
- Add builtin_interaction function to access NPC model interaction field
- Add interaction validation checks in interaction.lua matching removed C++ handlers
- Add condition checks for buy/sell handlers (sell size, buy has_value)
- Apply UTF8 conversion for string values in generated const_map code
- Fix BUY_PRICE regex to require '?쇰쭏?? keyword
- Update const.xlsx data
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB4FF51C-BA1E-430E-BDE5-D49C6A93FC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6148808-9FDD-4027-A117-EB626C3A7A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="regex" sheetId="1" r:id="rId1"/>
@@ -109,9 +109,6 @@
     <t>(?:뭐|뭘|무엇을|무얼)\\s*(?:사니|사냐|사고\\s*(?:있니|있냐))</t>
   </si>
   <si>
-    <t>(?P&lt;name&gt;\\S+)\\s+(?:얼마에\\s?)?사(?:니|냐)</t>
-  </si>
-  <si>
     <t>(?:돈|금전)\\s*얼마(?:나)?\\s*맡(?:아두)?고\\s*있(?:니|냐)</t>
   </si>
   <si>
@@ -327,6 +324,10 @@
   </si>
   <si>
     <t>listing_limit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(?P&lt;name&gt;\\S+)\\s+얼마에\\s?사(?:니|냐)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -410,7 +411,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -426,7 +427,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -812,7 +813,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>0</v>
@@ -826,7 +827,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>0</v>
@@ -877,7 +878,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -891,7 +892,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>24</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -905,7 +906,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -919,7 +920,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -933,7 +934,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -947,35 +948,35 @@
         <v>1</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -996,13 +997,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="D1" s="3">
         <v>6.9444444444444447E-4</v>
@@ -1025,13 +1026,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>53</v>
       </c>
       <c r="D1" s="4">
         <v>0.05</v>
@@ -1039,27 +1040,27 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D3" s="3">
         <v>2.0833333333333332E-2</v>
@@ -1082,86 +1083,86 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="D6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1180,16 +1181,16 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1209,27 +1210,27 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>79</v>
       </c>
       <c r="D2" s="5">
         <v>20</v>
@@ -1237,27 +1238,27 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D4" s="5">
         <v>5</v>
@@ -1282,58 +1283,58 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1353,13 +1354,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D1" s="2">
         <v>20</v>
@@ -1367,13 +1368,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D2" s="2">
         <v>20</v>
@@ -1398,7 +1399,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1407,12 +1408,12 @@
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
@@ -1421,12 +1422,12 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>0</v>
@@ -1435,21 +1436,21 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
script: remove regex tables from model and scripts
- Remove REGEX enum/const definitions from generated model outputs
- Delete enum.regex table and sync const/model artifacts
- Keep chat regex definitions in interaction.lua
- Clean bulk Lua script header/trailing comments in npc/item/spell files
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6148808-9FDD-4027-A117-EB626C3A7A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1D0F42-3426-48B2-A18F-2A43CF63E1F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
-    <sheet name="regex" sheetId="1" r:id="rId1"/>
-    <sheet name="time" sheetId="5" r:id="rId2"/>
-    <sheet name="death_penalty" sheetId="6" r:id="rId3"/>
-    <sheet name="item" sheetId="4" r:id="rId4"/>
-    <sheet name="mob" sheetId="3" r:id="rId5"/>
-    <sheet name="marketplace" sheetId="10" r:id="rId6"/>
-    <sheet name="clan" sheetId="7" r:id="rId7"/>
-    <sheet name="mail" sheetId="8" r:id="rId8"/>
-    <sheet name="script" sheetId="9" r:id="rId9"/>
+    <sheet name="time" sheetId="5" r:id="rId1"/>
+    <sheet name="death_penalty" sheetId="6" r:id="rId2"/>
+    <sheet name="item" sheetId="4" r:id="rId3"/>
+    <sheet name="mob" sheetId="3" r:id="rId4"/>
+    <sheet name="marketplace" sheetId="10" r:id="rId5"/>
+    <sheet name="clan" sheetId="7" r:id="rId6"/>
+    <sheet name="mail" sheetId="8" r:id="rId7"/>
+    <sheet name="script" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -33,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="49">
   <si>
     <t>server</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -43,84 +42,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>SELL</t>
-  </si>
-  <si>
-    <t>BUY</t>
-  </si>
-  <si>
-    <t>REPAIR</t>
-  </si>
-  <si>
-    <t>DEPOSIT_MONEY</t>
-  </si>
-  <si>
-    <t>WITHDRAW_MONEY</t>
-  </si>
-  <si>
-    <t>SELL_LIST</t>
-  </si>
-  <si>
-    <t>BUY_LIST</t>
-  </si>
-  <si>
-    <t>SELL_PRICE</t>
-  </si>
-  <si>
-    <t>BUY_PRICE</t>
-  </si>
-  <si>
-    <t>DEPOSITED_MONEY</t>
-  </si>
-  <si>
-    <t>RENAME_WEAPON</t>
-  </si>
-  <si>
-    <t>HOLD_ITEM_LIST</t>
-  </si>
-  <si>
-    <t>HOLD_ITEM_COUNT</t>
-  </si>
-  <si>
-    <t>(?P&lt;name&gt;\\S+)\\s+(?:(?:(?:(?P&lt;count&gt;\\d+)개)|(?P&lt;all&gt;다|전부))\\s+)?(?:판다|팜|팔게)</t>
-  </si>
-  <si>
-    <t>(?P&lt;name&gt;\\S+)\\s+(?:(?:(?:(?P&lt;count&gt;\\d+)개))\\s+)?(?:산다|줘|주세요)</t>
-  </si>
-  <si>
-    <t>(((?P&lt;all&gt;전부|모두|다)|(?P&lt;name&gt;\\S+))\\s+?(?:고쳐|수리\\s*해))\\s*줘</t>
-  </si>
-  <si>
-    <t>(?:돈|금전)\\s+(?:(?P&lt;money&gt;\\d+)(?:원|전)|(?P&lt;all&gt;(?:전부)?(?:\\s*다)?))\\s+맡아\\s*(?:줘|놔|주세요)</t>
-  </si>
-  <si>
-    <t>(?:돈|금전)\\s+(?:(?P&lt;money&gt;\\d+)(?:원|전)|(?P&lt;all&gt;(?:전부)?(?:\\s*다)?))\\s+돌려\\s*(?:줘|놔|주세요)</t>
-  </si>
-  <si>
-    <t>(?P&lt;name&gt;\\S+)\\s+(?:(?:(?P&lt;count&gt;\\d+)(?:개)|(?P&lt;all&gt;(?:전부)?(?:\\s*다)?))\\s+)?맡아\\s*(?:줘|놔|주세요)</t>
-  </si>
-  <si>
-    <t>(?P&lt;name&gt;\\S+)\\s+(?:(?:(?P&lt;count&gt;\\d+)(?:개)|(?P&lt;all&gt;(?:전부)?(?:\\s*다)?))\\s+)?돌려\\s*(?:줘|놔|주세요)</t>
-  </si>
-  <si>
-    <t>(?:뭐|뭘|무엇을|무얼)\\s*(?:파니|파냐|팔고\\s*(?:있니|있냐))</t>
-  </si>
-  <si>
-    <t>(?:뭐|뭘|무엇을|무얼)\\s*(?:사니|사냐|사고\\s*(?:있니|있냐))</t>
-  </si>
-  <si>
-    <t>(?:돈|금전)\\s*얼마(?:나)?\\s*맡(?:아두)?고\\s*있(?:니|냐)</t>
-  </si>
-  <si>
-    <t>(?P&lt;weapon&gt;\\S+?)?(?:의|$)?\\s+이름을\\s+(?P&lt;name&gt;\\S+?)?(?:으|$)?로\\s+명명</t>
-  </si>
-  <si>
-    <t>(?:뭐|뭘|무엇을|무얼)\\s*맡고\\s*(?:있니|있냐)</t>
-  </si>
-  <si>
-    <t>(?P&lt;name&gt;\\S+)\\s+(?:몇\\s*개|얼마나)\\s*맡고\\s*있(?:니|냐)</t>
-  </si>
-  <si>
     <t>$mob</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -177,24 +98,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>REVIVE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>살려(?:(?P&lt;ok&gt;(?:주세요|주십시오))|(?P&lt;no&gt;(?:줘|내|라|주소)))</t>
-  </si>
-  <si>
-    <t>APPRECIATE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>(감사합니다|고맙습니다)</t>
-  </si>
-  <si>
-    <t>(?P&lt;name&gt;\\S+)\\s+얼마(?:(?:(?:니|야|임|냐|에\\s*파(?:니|냐)))|(?:파(?:니|냐|)))</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>ANNOUNCE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -223,14 +126,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>STORE_ITEM</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RETRIEVE_ITEM</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>CLAN_ROLE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -324,10 +219,6 @@
   </si>
   <si>
     <t>listing_limit</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>(?P&lt;name&gt;\\S+)\\s+얼마에\\s?사(?:니|냐)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -722,271 +613,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE7A1E07-EEF2-4E86-80A0-A85D709C37E7}">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="94.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9" style="1"/>
-    <col min="11" max="11" width="22.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="26.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="31.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{651ECB05-F27B-4A03-ACAD-248FC1FCF2EE}">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -997,13 +623,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="D1" s="3">
         <v>6.9444444444444447E-4</v>
@@ -1015,7 +641,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EEF8597-1DC6-469B-AB8E-88EA492E15DC}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1026,13 +652,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="D1" s="4">
         <v>0.05</v>
@@ -1040,27 +666,27 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="D3" s="3">
         <v>2.0833333333333332E-2</v>
@@ -1072,7 +698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B64BF8E-904C-4727-916B-44450F4B2927}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1083,86 +709,86 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1171,7 +797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71AA2139-4412-4459-975E-C6152019FA56}">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1181,16 +807,16 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1199,7 +825,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5478E627-A9E2-4CC4-9690-22D3BFBD3A42}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1210,27 +836,27 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="D2" s="5">
         <v>20</v>
@@ -1238,27 +864,27 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>81</v>
+        <v>48</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="D4" s="5">
         <v>5</v>
@@ -1270,7 +896,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5047E650-3765-47B1-A7FE-DA9F7A8550D3}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1283,58 +909,58 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>64</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1343,7 +969,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25A28286-3AEF-42D4-85D1-723078A774E6}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1354,13 +980,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="D1" s="2">
         <v>20</v>
@@ -1368,13 +994,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="D2" s="2">
         <v>20</v>
@@ -1386,7 +1012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49D81130-7A86-4FD0-BE88-6F2B508E57F2}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1399,7 +1025,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1408,12 +1034,12 @@
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
@@ -1422,12 +1048,12 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>70</v>
+        <v>37</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>0</v>
@@ -1436,12 +1062,12 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>0</v>
@@ -1450,7 +1076,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: use lower snake_case for Lua hook names
- Rename ON_* export keys and call sites to on_*
- Update F1/F2 and schedule func constants in model and tables
- Remove obsolete skill test audit markdown
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1D0F42-3426-48B2-A18F-2A43CF63E1F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8129C2D3-CCD1-4121-B3BF-D4904823272D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="time" sheetId="5" r:id="rId1"/>
@@ -182,18 +182,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ON_F1_EVENT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>F2_EVENT_FUNC</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ON_F2_EVENT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>0.05</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -219,6 +211,14 @@
   </si>
   <si>
     <t>listing_limit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>on_f1_event</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>on_f2_event</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -836,7 +836,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -845,18 +845,18 @@
         <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D2" s="5">
         <v>20</v>
@@ -864,7 +864,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>0</v>
@@ -873,18 +873,18 @@
         <v>19</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D4" s="5">
         <v>5</v>
@@ -1062,12 +1062,12 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>